<commit_message>
Updates in.json format - rerun all extracts
</commit_message>
<xml_diff>
--- a/submission_guidelines/docs/RSETraining AI Project.xlsx
+++ b/submission_guidelines/docs/RSETraining AI Project.xlsx
@@ -1,20 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/magd4194/SoftwareEngineeringCourse/oxford-apc-finder/submission_guidelines/docs/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F43627B2-BB32-8E4A-96F6-1443DC97CC05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Journals" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="JSON Format and Rules" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Example JSON output" sheetId="4" r:id="rId8"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Journals" sheetId="2" r:id="rId2"/>
+    <sheet name="JSON Format and Rules" sheetId="3" r:id="rId3"/>
+    <sheet name="Example JSON output" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="309">
   <si>
     <t>Journal</t>
   </si>
@@ -324,21 +333,30 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://annals.math.princeton.edu/submission-guidelines</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
         <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">; </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://mirror.apps.cam.ac.uk/pub/tex-archive/macros/latex/contrib/aomart/aomart.pdf</t>
     </r>
@@ -610,43 +628,68 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/jlms/peerreview</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
         <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">; </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/jlms/submission</t>
     </r>
     <r>
-      <rPr/>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/jlms#submitting-to-the-journal</t>
     </r>
     <r>
-      <rPr/>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/policies/ethicalpolicy</t>
     </r>
@@ -717,21 +760,30 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://msp.org/gt/about/journal/about.html</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
         <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://msp.org/gt/about/journal/submissions.html</t>
     </r>
@@ -853,43 +905,68 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/jlms/peerreview</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
         <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">; </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/jlms/submission</t>
     </r>
     <r>
-      <rPr/>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/jlms#submitting-to-the-journal</t>
     </r>
     <r>
-      <rPr/>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://www.lms.ac.uk/publications/policies/ethicalpolicy</t>
     </r>
@@ -1058,98 +1135,139 @@
   </si>
   <si>
     <t>Universe</t>
+  </si>
+  <si>
+    <t>Perspectives in Ecology and Conservation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="17">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="19">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="&quot;Arial Unicode MS&quot;"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="8"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="8"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF6AA84F"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF4A86E8"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1157,103 +1275,68 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="19">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1443,33 +1526,36 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AG57"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="129.5"/>
-    <col customWidth="1" min="2" max="2" width="48.63"/>
-    <col customWidth="1" min="4" max="4" width="17.75"/>
-    <col customWidth="1" min="5" max="5" width="23.63"/>
-    <col customWidth="1" min="6" max="6" width="33.63"/>
-    <col customWidth="1" min="7" max="7" width="19.63"/>
-    <col customWidth="1" min="8" max="8" width="22.13"/>
-    <col customWidth="1" min="9" max="9" width="23.38"/>
-    <col customWidth="1" min="10" max="10" width="16.13"/>
-    <col customWidth="1" min="11" max="11" width="22.5"/>
-    <col customWidth="1" min="12" max="12" width="17.63"/>
-    <col customWidth="1" min="14" max="14" width="23.38"/>
-    <col customWidth="1" min="15" max="15" width="43.13"/>
-    <col customWidth="1" min="17" max="17" width="22.75"/>
+    <col min="1" max="1" width="129.5" customWidth="1"/>
+    <col min="2" max="2" width="48.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="23.6640625" customWidth="1"/>
+    <col min="6" max="6" width="33.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" customWidth="1"/>
+    <col min="8" max="8" width="22.1640625" customWidth="1"/>
+    <col min="9" max="9" width="23.33203125" customWidth="1"/>
+    <col min="10" max="10" width="16.1640625" customWidth="1"/>
+    <col min="11" max="11" width="22.5" customWidth="1"/>
+    <col min="12" max="12" width="17.6640625" customWidth="1"/>
+    <col min="14" max="14" width="23.33203125" customWidth="1"/>
+    <col min="15" max="15" width="43.1640625" customWidth="1"/>
+    <col min="17" max="17" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:33">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1527,600 +1613,598 @@
       <c r="S1" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8"/>
-      <c r="AB1" s="8"/>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="s">
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
+      <c r="Z1" s="7"/>
+      <c r="AA1" s="7"/>
+      <c r="AB1" s="7"/>
+      <c r="AC1" s="7"/>
+      <c r="AD1" s="7"/>
+      <c r="AE1" s="7"/>
+      <c r="AF1" s="7"/>
+      <c r="AG1" s="7"/>
+    </row>
+    <row r="2" spans="1:33">
+      <c r="A2" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="Q2" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:33">
+      <c r="A3" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="L3" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="S3" s="9" t="s">
+      <c r="S3" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:33">
+      <c r="A4" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="L4" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="N4" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="O4" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="P4" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="Q4" s="9" t="s">
+      <c r="Q4" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:33">
+      <c r="A5" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="L5" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="N5" s="12" t="s">
+      <c r="N5" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="O5" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="P5" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="Q5" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="12" t="s">
+    <row r="6" spans="1:33">
+      <c r="A6" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="L6" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="N6" s="9" t="s">
+      <c r="N6" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="P6" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="12" t="s">
+    <row r="7" spans="1:33">
+      <c r="A7" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="11" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:33">
+      <c r="A8" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="L8" s="9" t="s">
+      <c r="L8" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="O8" s="9" t="s">
+      <c r="O8" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="P8" s="9" t="s">
+      <c r="P8" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="Q8" s="9" t="s">
+      <c r="Q8" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="S8" s="9" t="s">
+      <c r="S8" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="s">
+    <row r="9" spans="1:33">
+      <c r="A9" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="11" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="s">
+    <row r="10" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A10" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="12" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="s">
+    <row r="11" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A11" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="12" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="s">
+    <row r="12" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A12" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="13" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A13" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="13" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="s">
+    <row r="14" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A14" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="13" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="s">
+    <row r="15" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A15" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="17" t="s">
+    <row r="16" spans="1:33" ht="15.75" customHeight="1">
+      <c r="B16" s="14" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="17" t="s">
+    <row r="17" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B17" s="14" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A18" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="12" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="12" t="s">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A19" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="15" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="12" t="s">
+    <row r="20" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A20" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="15" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="s">
+    <row r="21" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A21" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="12" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="17" t="s">
+    <row r="22" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B22" s="14" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="17" t="s">
+    <row r="23" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B23" s="14" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="17" t="s">
+    <row r="24" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B24" s="14" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="17" t="s">
+    <row r="25" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B25" s="14" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="17" t="s">
+    <row r="26" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B26" s="14" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="17" t="s">
+    <row r="27" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B27" s="14" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B28" s="14" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B29" s="14" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="17" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="17" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="17" t="s">
+    <row r="30" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B30" s="14" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="17" t="s">
+    <row r="31" spans="1:2" ht="15.75" customHeight="1">
+      <c r="B31" s="14" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="s">
+    <row r="32" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A32" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="15" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="s">
+    <row r="33" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A33" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="15" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="12" t="s">
+    <row r="34" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A34" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="B34" s="19" t="s">
+      <c r="B34" s="15" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="12" t="s">
+    <row r="35" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A35" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="B35" s="19" t="s">
+      <c r="B35" s="15" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="12" t="s">
+    <row r="36" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A36" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="B36" s="19" t="s">
+      <c r="B36" s="15" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A37" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="B37" s="19" t="s">
+      <c r="B37" s="15" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="12" t="s">
+    <row r="38" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A38" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="B38" s="19" t="s">
+      <c r="B38" s="15" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="10" t="s">
+    <row r="39" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A39" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="B39" s="19" t="s">
+      <c r="B39" s="15" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="12" t="s">
+    <row r="40" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A40" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="B40" s="19" t="s">
+      <c r="B40" s="15" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="12" t="s">
+    <row r="41" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A41" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="B41" s="19" t="s">
+      <c r="B41" s="15" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="20"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="20"/>
-    </row>
-    <row r="51">
-      <c r="B51" s="20"/>
-    </row>
-    <row r="52">
-      <c r="B52" s="20"/>
-    </row>
-    <row r="53">
-      <c r="B53" s="20"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="20"/>
-    </row>
-    <row r="55">
-      <c r="B55" s="20"/>
-    </row>
-    <row r="56">
-      <c r="B56" s="20"/>
-    </row>
-    <row r="57">
-      <c r="B57" s="20"/>
+    <row r="49" spans="2:2" ht="13">
+      <c r="B49" s="16"/>
+    </row>
+    <row r="50" spans="2:2" ht="13">
+      <c r="B50" s="16"/>
+    </row>
+    <row r="51" spans="2:2" ht="13">
+      <c r="B51" s="16"/>
+    </row>
+    <row r="52" spans="2:2" ht="13">
+      <c r="B52" s="16"/>
+    </row>
+    <row r="53" spans="2:2" ht="13">
+      <c r="B53" s="16"/>
+    </row>
+    <row r="54" spans="2:2" ht="13">
+      <c r="B54" s="16"/>
+    </row>
+    <row r="55" spans="2:2" ht="13">
+      <c r="B55" s="16"/>
+    </row>
+    <row r="56" spans="2:2" ht="13">
+      <c r="B56" s="16"/>
+    </row>
+    <row r="57" spans="2:2" ht="13">
+      <c r="B57" s="16"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A2"/>
-    <hyperlink r:id="rId2" ref="N2"/>
-    <hyperlink r:id="rId3" ref="A3"/>
-    <hyperlink r:id="rId4" ref="A4"/>
-    <hyperlink r:id="rId5" ref="N4"/>
-    <hyperlink r:id="rId6" ref="A5"/>
-    <hyperlink r:id="rId7" ref="N5"/>
-    <hyperlink r:id="rId8" location="submit" ref="A6"/>
-    <hyperlink r:id="rId9" ref="A7"/>
-    <hyperlink r:id="rId10" ref="A8"/>
-    <hyperlink r:id="rId11" ref="A9"/>
-    <hyperlink r:id="rId12" ref="A10"/>
-    <hyperlink r:id="rId13" ref="A11"/>
-    <hyperlink r:id="rId14" ref="A12"/>
-    <hyperlink r:id="rId15" ref="A13"/>
-    <hyperlink r:id="rId16" ref="A14"/>
-    <hyperlink r:id="rId17" ref="A15"/>
-    <hyperlink r:id="rId18" ref="A18"/>
-    <hyperlink r:id="rId19" ref="A19"/>
-    <hyperlink r:id="rId20" ref="A20"/>
-    <hyperlink r:id="rId21" ref="A21"/>
-    <hyperlink r:id="rId22" ref="A32"/>
-    <hyperlink r:id="rId23" ref="A33"/>
-    <hyperlink r:id="rId24" ref="A34"/>
-    <hyperlink r:id="rId25" ref="A35"/>
-    <hyperlink r:id="rId26" ref="A36"/>
-    <hyperlink r:id="rId27" ref="A37"/>
-    <hyperlink r:id="rId28" ref="A38"/>
-    <hyperlink r:id="rId29" ref="A39"/>
-    <hyperlink r:id="rId30" ref="A40"/>
-    <hyperlink r:id="rId31" ref="A41"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="A4" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N4" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="A5" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="A6" r:id="rId8" location="submit" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="A7" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="A8" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="A9" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="A10" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="A11" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="A12" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="A13" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="A14" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="A15" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="A18" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="A19" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="A20" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="A21" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="A32" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="A33" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="A34" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="A35" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="A36" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="A37" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="A38" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="A39" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="A40" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="A41" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
   </hyperlinks>
-  <drawing r:id="rId32"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:AL1000"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="3" width="12.25"/>
-    <col customWidth="1" min="4" max="4" width="16.63"/>
-    <col customWidth="1" min="5" max="5" width="35.0"/>
-    <col customWidth="1" min="6" max="7" width="12.25"/>
-    <col customWidth="1" min="8" max="8" width="17.5"/>
-    <col customWidth="1" min="9" max="9" width="16.63"/>
-    <col customWidth="1" min="10" max="10" width="15.75"/>
-    <col customWidth="1" min="11" max="11" width="16.63"/>
-    <col customWidth="1" min="12" max="12" width="22.75"/>
-    <col customWidth="1" min="13" max="13" width="21.88"/>
-    <col customWidth="1" min="14" max="14" width="14.88"/>
-    <col customWidth="1" min="15" max="15" width="21.0"/>
-    <col customWidth="1" min="16" max="16" width="13.13"/>
-    <col customWidth="1" min="17" max="17" width="19.25"/>
-    <col customWidth="1" min="18" max="18" width="14.0"/>
-    <col customWidth="1" min="19" max="20" width="12.25"/>
-    <col customWidth="1" min="21" max="21" width="16.63"/>
-    <col customWidth="1" min="22" max="22" width="22.75"/>
-    <col customWidth="1" min="23" max="23" width="21.88"/>
-    <col customWidth="1" min="24" max="24" width="35.0"/>
-    <col customWidth="1" min="25" max="25" width="12.25"/>
-    <col customWidth="1" min="26" max="26" width="18.38"/>
-    <col customWidth="1" min="27" max="28" width="21.0"/>
-    <col customWidth="1" min="29" max="29" width="21.88"/>
-    <col customWidth="1" min="30" max="30" width="25.38"/>
-    <col customWidth="1" min="31" max="31" width="22.75"/>
-    <col customWidth="1" min="32" max="32" width="16.63"/>
-    <col customWidth="1" min="33" max="33" width="13.13"/>
-    <col customWidth="1" min="34" max="35" width="14.88"/>
-    <col customWidth="1" min="36" max="36" width="17.5"/>
-    <col customWidth="1" min="37" max="38" width="12.25"/>
+    <col min="1" max="3" width="12.1640625" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="35" customWidth="1"/>
+    <col min="6" max="7" width="12.1640625" customWidth="1"/>
+    <col min="8" max="8" width="17.5" customWidth="1"/>
+    <col min="9" max="9" width="16.6640625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="21" customWidth="1"/>
+    <col min="16" max="16" width="13.1640625" customWidth="1"/>
+    <col min="17" max="17" width="19.1640625" customWidth="1"/>
+    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="19" max="20" width="12.1640625" customWidth="1"/>
+    <col min="21" max="21" width="16.6640625" customWidth="1"/>
+    <col min="22" max="22" width="22.6640625" customWidth="1"/>
+    <col min="23" max="23" width="21.83203125" customWidth="1"/>
+    <col min="24" max="24" width="35" customWidth="1"/>
+    <col min="25" max="25" width="12.1640625" customWidth="1"/>
+    <col min="26" max="26" width="18.33203125" customWidth="1"/>
+    <col min="27" max="28" width="21" customWidth="1"/>
+    <col min="29" max="29" width="21.83203125" customWidth="1"/>
+    <col min="30" max="30" width="25.33203125" customWidth="1"/>
+    <col min="31" max="31" width="22.6640625" customWidth="1"/>
+    <col min="32" max="32" width="16.6640625" customWidth="1"/>
+    <col min="33" max="33" width="13.1640625" customWidth="1"/>
+    <col min="34" max="35" width="14.83203125" customWidth="1"/>
+    <col min="36" max="36" width="17.5" customWidth="1"/>
+    <col min="37" max="38" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:38" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2236,7 +2320,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:38" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>43</v>
       </c>
@@ -2316,10 +2400,10 @@
         <v>63</v>
       </c>
       <c r="AA2" s="1">
-        <v>2500.0</v>
+        <v>2500</v>
       </c>
       <c r="AB2" s="1">
-        <v>4300.0</v>
+        <v>4300</v>
       </c>
       <c r="AC2" s="1" t="s">
         <v>76</v>
@@ -2337,7 +2421,7 @@
         <v>80</v>
       </c>
       <c r="AH2" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="AI2" s="1" t="s">
         <v>82</v>
@@ -2352,7 +2436,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:38" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>43</v>
       </c>
@@ -2435,7 +2519,7 @@
         <v>70</v>
       </c>
       <c r="AB3" s="1">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="AC3" s="1" t="s">
         <v>76</v>
@@ -2453,7 +2537,7 @@
         <v>70</v>
       </c>
       <c r="AH3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>100</v>
@@ -2468,7 +2552,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:38" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>43</v>
       </c>
@@ -2551,7 +2635,7 @@
         <v>70</v>
       </c>
       <c r="AB4" s="1">
-        <v>1200.0</v>
+        <v>1200</v>
       </c>
       <c r="AC4" s="1" t="s">
         <v>76</v>
@@ -2569,7 +2653,7 @@
         <v>119</v>
       </c>
       <c r="AH4" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>120</v>
@@ -2584,7 +2668,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:38" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
@@ -2700,7 +2784,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:38" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>43</v>
       </c>
@@ -2816,7 +2900,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:38" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>43</v>
       </c>
@@ -2932,7 +3016,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:38" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>43</v>
       </c>
@@ -3048,1007 +3132,981 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
-    <row r="1000"/>
+    <row r="46" ht="13"/>
+    <row r="47" ht="13"/>
+    <row r="48" ht="13"/>
+    <row r="49" ht="13"/>
+    <row r="50" ht="13"/>
+    <row r="51" ht="13"/>
+    <row r="52" ht="13"/>
+    <row r="53" ht="13"/>
+    <row r="54" ht="13"/>
+    <row r="55" ht="13"/>
+    <row r="56" ht="13"/>
+    <row r="57" ht="13"/>
+    <row r="58" ht="13"/>
+    <row r="59" ht="13"/>
+    <row r="60" ht="13"/>
+    <row r="61" ht="13"/>
+    <row r="62" ht="13"/>
+    <row r="63" ht="13"/>
+    <row r="64" ht="13"/>
+    <row r="65" ht="13"/>
+    <row r="66" ht="13"/>
+    <row r="67" ht="13"/>
+    <row r="68" ht="13"/>
+    <row r="69" ht="13"/>
+    <row r="70" ht="13"/>
+    <row r="71" ht="13"/>
+    <row r="72" ht="13"/>
+    <row r="73" ht="13"/>
+    <row r="74" ht="13"/>
+    <row r="75" ht="13"/>
+    <row r="76" ht="13"/>
+    <row r="77" ht="13"/>
+    <row r="78" ht="13"/>
+    <row r="79" ht="13"/>
+    <row r="80" ht="13"/>
+    <row r="81" ht="13"/>
+    <row r="82" ht="13"/>
+    <row r="83" ht="13"/>
+    <row r="84" ht="13"/>
+    <row r="85" ht="13"/>
+    <row r="86" ht="13"/>
+    <row r="87" ht="13"/>
+    <row r="88" ht="13"/>
+    <row r="89" ht="13"/>
+    <row r="90" ht="13"/>
+    <row r="91" ht="13"/>
+    <row r="92" ht="13"/>
+    <row r="93" ht="13"/>
+    <row r="94" ht="13"/>
+    <row r="95" ht="13"/>
+    <row r="96" ht="13"/>
+    <row r="97" ht="13"/>
+    <row r="98" ht="13"/>
+    <row r="99" ht="13"/>
+    <row r="100" ht="13"/>
+    <row r="101" ht="13"/>
+    <row r="102" ht="13"/>
+    <row r="103" ht="13"/>
+    <row r="104" ht="13"/>
+    <row r="105" ht="13"/>
+    <row r="106" ht="13"/>
+    <row r="107" ht="13"/>
+    <row r="108" ht="13"/>
+    <row r="109" ht="13"/>
+    <row r="110" ht="13"/>
+    <row r="111" ht="13"/>
+    <row r="112" ht="13"/>
+    <row r="113" ht="13"/>
+    <row r="114" ht="13"/>
+    <row r="115" ht="13"/>
+    <row r="116" ht="13"/>
+    <row r="117" ht="13"/>
+    <row r="118" ht="13"/>
+    <row r="119" ht="13"/>
+    <row r="120" ht="13"/>
+    <row r="121" ht="13"/>
+    <row r="122" ht="13"/>
+    <row r="123" ht="13"/>
+    <row r="124" ht="13"/>
+    <row r="125" ht="13"/>
+    <row r="126" ht="13"/>
+    <row r="127" ht="13"/>
+    <row r="128" ht="13"/>
+    <row r="129" ht="13"/>
+    <row r="130" ht="13"/>
+    <row r="131" ht="13"/>
+    <row r="132" ht="13"/>
+    <row r="133" ht="13"/>
+    <row r="134" ht="13"/>
+    <row r="135" ht="13"/>
+    <row r="136" ht="13"/>
+    <row r="137" ht="13"/>
+    <row r="138" ht="13"/>
+    <row r="139" ht="13"/>
+    <row r="140" ht="13"/>
+    <row r="141" ht="13"/>
+    <row r="142" ht="13"/>
+    <row r="143" ht="13"/>
+    <row r="144" ht="13"/>
+    <row r="145" ht="13"/>
+    <row r="146" ht="13"/>
+    <row r="147" ht="13"/>
+    <row r="148" ht="13"/>
+    <row r="149" ht="13"/>
+    <row r="150" ht="13"/>
+    <row r="151" ht="13"/>
+    <row r="152" ht="13"/>
+    <row r="153" ht="13"/>
+    <row r="154" ht="13"/>
+    <row r="155" ht="13"/>
+    <row r="156" ht="13"/>
+    <row r="157" ht="13"/>
+    <row r="158" ht="13"/>
+    <row r="159" ht="13"/>
+    <row r="160" ht="13"/>
+    <row r="161" ht="13"/>
+    <row r="162" ht="13"/>
+    <row r="163" ht="13"/>
+    <row r="164" ht="13"/>
+    <row r="165" ht="13"/>
+    <row r="166" ht="13"/>
+    <row r="167" ht="13"/>
+    <row r="168" ht="13"/>
+    <row r="169" ht="13"/>
+    <row r="170" ht="13"/>
+    <row r="171" ht="13"/>
+    <row r="172" ht="13"/>
+    <row r="173" ht="13"/>
+    <row r="174" ht="13"/>
+    <row r="175" ht="13"/>
+    <row r="176" ht="13"/>
+    <row r="177" ht="13"/>
+    <row r="178" ht="13"/>
+    <row r="179" ht="13"/>
+    <row r="180" ht="13"/>
+    <row r="181" ht="13"/>
+    <row r="182" ht="13"/>
+    <row r="183" ht="13"/>
+    <row r="184" ht="13"/>
+    <row r="185" ht="13"/>
+    <row r="186" ht="13"/>
+    <row r="187" ht="13"/>
+    <row r="188" ht="13"/>
+    <row r="189" ht="13"/>
+    <row r="190" ht="13"/>
+    <row r="191" ht="13"/>
+    <row r="192" ht="13"/>
+    <row r="193" ht="13"/>
+    <row r="194" ht="13"/>
+    <row r="195" ht="13"/>
+    <row r="196" ht="13"/>
+    <row r="197" ht="13"/>
+    <row r="198" ht="13"/>
+    <row r="199" ht="13"/>
+    <row r="200" ht="13"/>
+    <row r="201" ht="13"/>
+    <row r="202" ht="13"/>
+    <row r="203" ht="13"/>
+    <row r="204" ht="13"/>
+    <row r="205" ht="13"/>
+    <row r="206" ht="13"/>
+    <row r="207" ht="13"/>
+    <row r="208" ht="13"/>
+    <row r="209" ht="13"/>
+    <row r="210" ht="13"/>
+    <row r="211" ht="13"/>
+    <row r="212" ht="13"/>
+    <row r="213" ht="13"/>
+    <row r="214" ht="13"/>
+    <row r="215" ht="13"/>
+    <row r="216" ht="13"/>
+    <row r="217" ht="13"/>
+    <row r="218" ht="13"/>
+    <row r="219" ht="13"/>
+    <row r="220" ht="13"/>
+    <row r="221" ht="13"/>
+    <row r="222" ht="13"/>
+    <row r="223" ht="13"/>
+    <row r="224" ht="13"/>
+    <row r="225" ht="13"/>
+    <row r="226" ht="13"/>
+    <row r="227" ht="13"/>
+    <row r="228" ht="13"/>
+    <row r="229" ht="13"/>
+    <row r="230" ht="13"/>
+    <row r="231" ht="13"/>
+    <row r="232" ht="13"/>
+    <row r="233" ht="13"/>
+    <row r="234" ht="13"/>
+    <row r="235" ht="13"/>
+    <row r="236" ht="13"/>
+    <row r="237" ht="13"/>
+    <row r="238" ht="13"/>
+    <row r="239" ht="13"/>
+    <row r="240" ht="13"/>
+    <row r="241" ht="13"/>
+    <row r="242" ht="13"/>
+    <row r="243" ht="13"/>
+    <row r="244" ht="13"/>
+    <row r="245" ht="13"/>
+    <row r="246" ht="13"/>
+    <row r="247" ht="13"/>
+    <row r="248" ht="13"/>
+    <row r="249" ht="13"/>
+    <row r="250" ht="13"/>
+    <row r="251" ht="13"/>
+    <row r="252" ht="13"/>
+    <row r="253" ht="13"/>
+    <row r="254" ht="13"/>
+    <row r="255" ht="13"/>
+    <row r="256" ht="13"/>
+    <row r="257" ht="13"/>
+    <row r="258" ht="13"/>
+    <row r="259" ht="13"/>
+    <row r="260" ht="13"/>
+    <row r="261" ht="13"/>
+    <row r="262" ht="13"/>
+    <row r="263" ht="13"/>
+    <row r="264" ht="13"/>
+    <row r="265" ht="13"/>
+    <row r="266" ht="13"/>
+    <row r="267" ht="13"/>
+    <row r="268" ht="13"/>
+    <row r="269" ht="13"/>
+    <row r="270" ht="13"/>
+    <row r="271" ht="13"/>
+    <row r="272" ht="13"/>
+    <row r="273" ht="13"/>
+    <row r="274" ht="13"/>
+    <row r="275" ht="13"/>
+    <row r="276" ht="13"/>
+    <row r="277" ht="13"/>
+    <row r="278" ht="13"/>
+    <row r="279" ht="13"/>
+    <row r="280" ht="13"/>
+    <row r="281" ht="13"/>
+    <row r="282" ht="13"/>
+    <row r="283" ht="13"/>
+    <row r="284" ht="13"/>
+    <row r="285" ht="13"/>
+    <row r="286" ht="13"/>
+    <row r="287" ht="13"/>
+    <row r="288" ht="13"/>
+    <row r="289" ht="13"/>
+    <row r="290" ht="13"/>
+    <row r="291" ht="13"/>
+    <row r="292" ht="13"/>
+    <row r="293" ht="13"/>
+    <row r="294" ht="13"/>
+    <row r="295" ht="13"/>
+    <row r="296" ht="13"/>
+    <row r="297" ht="13"/>
+    <row r="298" ht="13"/>
+    <row r="299" ht="13"/>
+    <row r="300" ht="13"/>
+    <row r="301" ht="13"/>
+    <row r="302" ht="13"/>
+    <row r="303" ht="13"/>
+    <row r="304" ht="13"/>
+    <row r="305" ht="13"/>
+    <row r="306" ht="13"/>
+    <row r="307" ht="13"/>
+    <row r="308" ht="13"/>
+    <row r="309" ht="13"/>
+    <row r="310" ht="13"/>
+    <row r="311" ht="13"/>
+    <row r="312" ht="13"/>
+    <row r="313" ht="13"/>
+    <row r="314" ht="13"/>
+    <row r="315" ht="13"/>
+    <row r="316" ht="13"/>
+    <row r="317" ht="13"/>
+    <row r="318" ht="13"/>
+    <row r="319" ht="13"/>
+    <row r="320" ht="13"/>
+    <row r="321" ht="13"/>
+    <row r="322" ht="13"/>
+    <row r="323" ht="13"/>
+    <row r="324" ht="13"/>
+    <row r="325" ht="13"/>
+    <row r="326" ht="13"/>
+    <row r="327" ht="13"/>
+    <row r="328" ht="13"/>
+    <row r="329" ht="13"/>
+    <row r="330" ht="13"/>
+    <row r="331" ht="13"/>
+    <row r="332" ht="13"/>
+    <row r="333" ht="13"/>
+    <row r="334" ht="13"/>
+    <row r="335" ht="13"/>
+    <row r="336" ht="13"/>
+    <row r="337" ht="13"/>
+    <row r="338" ht="13"/>
+    <row r="339" ht="13"/>
+    <row r="340" ht="13"/>
+    <row r="341" ht="13"/>
+    <row r="342" ht="13"/>
+    <row r="343" ht="13"/>
+    <row r="344" ht="13"/>
+    <row r="345" ht="13"/>
+    <row r="346" ht="13"/>
+    <row r="347" ht="13"/>
+    <row r="348" ht="13"/>
+    <row r="349" ht="13"/>
+    <row r="350" ht="13"/>
+    <row r="351" ht="13"/>
+    <row r="352" ht="13"/>
+    <row r="353" ht="13"/>
+    <row r="354" ht="13"/>
+    <row r="355" ht="13"/>
+    <row r="356" ht="13"/>
+    <row r="357" ht="13"/>
+    <row r="358" ht="13"/>
+    <row r="359" ht="13"/>
+    <row r="360" ht="13"/>
+    <row r="361" ht="13"/>
+    <row r="362" ht="13"/>
+    <row r="363" ht="13"/>
+    <row r="364" ht="13"/>
+    <row r="365" ht="13"/>
+    <row r="366" ht="13"/>
+    <row r="367" ht="13"/>
+    <row r="368" ht="13"/>
+    <row r="369" ht="13"/>
+    <row r="370" ht="13"/>
+    <row r="371" ht="13"/>
+    <row r="372" ht="13"/>
+    <row r="373" ht="13"/>
+    <row r="374" ht="13"/>
+    <row r="375" ht="13"/>
+    <row r="376" ht="13"/>
+    <row r="377" ht="13"/>
+    <row r="378" ht="13"/>
+    <row r="379" ht="13"/>
+    <row r="380" ht="13"/>
+    <row r="381" ht="13"/>
+    <row r="382" ht="13"/>
+    <row r="383" ht="13"/>
+    <row r="384" ht="13"/>
+    <row r="385" ht="13"/>
+    <row r="386" ht="13"/>
+    <row r="387" ht="13"/>
+    <row r="388" ht="13"/>
+    <row r="389" ht="13"/>
+    <row r="390" ht="13"/>
+    <row r="391" ht="13"/>
+    <row r="392" ht="13"/>
+    <row r="393" ht="13"/>
+    <row r="394" ht="13"/>
+    <row r="395" ht="13"/>
+    <row r="396" ht="13"/>
+    <row r="397" ht="13"/>
+    <row r="398" ht="13"/>
+    <row r="399" ht="13"/>
+    <row r="400" ht="13"/>
+    <row r="401" ht="13"/>
+    <row r="402" ht="13"/>
+    <row r="403" ht="13"/>
+    <row r="404" ht="13"/>
+    <row r="405" ht="13"/>
+    <row r="406" ht="13"/>
+    <row r="407" ht="13"/>
+    <row r="408" ht="13"/>
+    <row r="409" ht="13"/>
+    <row r="410" ht="13"/>
+    <row r="411" ht="13"/>
+    <row r="412" ht="13"/>
+    <row r="413" ht="13"/>
+    <row r="414" ht="13"/>
+    <row r="415" ht="13"/>
+    <row r="416" ht="13"/>
+    <row r="417" ht="13"/>
+    <row r="418" ht="13"/>
+    <row r="419" ht="13"/>
+    <row r="420" ht="13"/>
+    <row r="421" ht="13"/>
+    <row r="422" ht="13"/>
+    <row r="423" ht="13"/>
+    <row r="424" ht="13"/>
+    <row r="425" ht="13"/>
+    <row r="426" ht="13"/>
+    <row r="427" ht="13"/>
+    <row r="428" ht="13"/>
+    <row r="429" ht="13"/>
+    <row r="430" ht="13"/>
+    <row r="431" ht="13"/>
+    <row r="432" ht="13"/>
+    <row r="433" ht="13"/>
+    <row r="434" ht="13"/>
+    <row r="435" ht="13"/>
+    <row r="436" ht="13"/>
+    <row r="437" ht="13"/>
+    <row r="438" ht="13"/>
+    <row r="439" ht="13"/>
+    <row r="440" ht="13"/>
+    <row r="441" ht="13"/>
+    <row r="442" ht="13"/>
+    <row r="443" ht="13"/>
+    <row r="444" ht="13"/>
+    <row r="445" ht="13"/>
+    <row r="446" ht="13"/>
+    <row r="447" ht="13"/>
+    <row r="448" ht="13"/>
+    <row r="449" ht="13"/>
+    <row r="450" ht="13"/>
+    <row r="451" ht="13"/>
+    <row r="452" ht="13"/>
+    <row r="453" ht="13"/>
+    <row r="454" ht="13"/>
+    <row r="455" ht="13"/>
+    <row r="456" ht="13"/>
+    <row r="457" ht="13"/>
+    <row r="458" ht="13"/>
+    <row r="459" ht="13"/>
+    <row r="460" ht="13"/>
+    <row r="461" ht="13"/>
+    <row r="462" ht="13"/>
+    <row r="463" ht="13"/>
+    <row r="464" ht="13"/>
+    <row r="465" ht="13"/>
+    <row r="466" ht="13"/>
+    <row r="467" ht="13"/>
+    <row r="468" ht="13"/>
+    <row r="469" ht="13"/>
+    <row r="470" ht="13"/>
+    <row r="471" ht="13"/>
+    <row r="472" ht="13"/>
+    <row r="473" ht="13"/>
+    <row r="474" ht="13"/>
+    <row r="475" ht="13"/>
+    <row r="476" ht="13"/>
+    <row r="477" ht="13"/>
+    <row r="478" ht="13"/>
+    <row r="479" ht="13"/>
+    <row r="480" ht="13"/>
+    <row r="481" ht="13"/>
+    <row r="482" ht="13"/>
+    <row r="483" ht="13"/>
+    <row r="484" ht="13"/>
+    <row r="485" ht="13"/>
+    <row r="486" ht="13"/>
+    <row r="487" ht="13"/>
+    <row r="488" ht="13"/>
+    <row r="489" ht="13"/>
+    <row r="490" ht="13"/>
+    <row r="491" ht="13"/>
+    <row r="492" ht="13"/>
+    <row r="493" ht="13"/>
+    <row r="494" ht="13"/>
+    <row r="495" ht="13"/>
+    <row r="496" ht="13"/>
+    <row r="497" ht="13"/>
+    <row r="498" ht="13"/>
+    <row r="499" ht="13"/>
+    <row r="500" ht="13"/>
+    <row r="501" ht="13"/>
+    <row r="502" ht="13"/>
+    <row r="503" ht="13"/>
+    <row r="504" ht="13"/>
+    <row r="505" ht="13"/>
+    <row r="506" ht="13"/>
+    <row r="507" ht="13"/>
+    <row r="508" ht="13"/>
+    <row r="509" ht="13"/>
+    <row r="510" ht="13"/>
+    <row r="511" ht="13"/>
+    <row r="512" ht="13"/>
+    <row r="513" ht="13"/>
+    <row r="514" ht="13"/>
+    <row r="515" ht="13"/>
+    <row r="516" ht="13"/>
+    <row r="517" ht="13"/>
+    <row r="518" ht="13"/>
+    <row r="519" ht="13"/>
+    <row r="520" ht="13"/>
+    <row r="521" ht="13"/>
+    <row r="522" ht="13"/>
+    <row r="523" ht="13"/>
+    <row r="524" ht="13"/>
+    <row r="525" ht="13"/>
+    <row r="526" ht="13"/>
+    <row r="527" ht="13"/>
+    <row r="528" ht="13"/>
+    <row r="529" ht="13"/>
+    <row r="530" ht="13"/>
+    <row r="531" ht="13"/>
+    <row r="532" ht="13"/>
+    <row r="533" ht="13"/>
+    <row r="534" ht="13"/>
+    <row r="535" ht="13"/>
+    <row r="536" ht="13"/>
+    <row r="537" ht="13"/>
+    <row r="538" ht="13"/>
+    <row r="539" ht="13"/>
+    <row r="540" ht="13"/>
+    <row r="541" ht="13"/>
+    <row r="542" ht="13"/>
+    <row r="543" ht="13"/>
+    <row r="544" ht="13"/>
+    <row r="545" ht="13"/>
+    <row r="546" ht="13"/>
+    <row r="547" ht="13"/>
+    <row r="548" ht="13"/>
+    <row r="549" ht="13"/>
+    <row r="550" ht="13"/>
+    <row r="551" ht="13"/>
+    <row r="552" ht="13"/>
+    <row r="553" ht="13"/>
+    <row r="554" ht="13"/>
+    <row r="555" ht="13"/>
+    <row r="556" ht="13"/>
+    <row r="557" ht="13"/>
+    <row r="558" ht="13"/>
+    <row r="559" ht="13"/>
+    <row r="560" ht="13"/>
+    <row r="561" ht="13"/>
+    <row r="562" ht="13"/>
+    <row r="563" ht="13"/>
+    <row r="564" ht="13"/>
+    <row r="565" ht="13"/>
+    <row r="566" ht="13"/>
+    <row r="567" ht="13"/>
+    <row r="568" ht="13"/>
+    <row r="569" ht="13"/>
+    <row r="570" ht="13"/>
+    <row r="571" ht="13"/>
+    <row r="572" ht="13"/>
+    <row r="573" ht="13"/>
+    <row r="574" ht="13"/>
+    <row r="575" ht="13"/>
+    <row r="576" ht="13"/>
+    <row r="577" ht="13"/>
+    <row r="578" ht="13"/>
+    <row r="579" ht="13"/>
+    <row r="580" ht="13"/>
+    <row r="581" ht="13"/>
+    <row r="582" ht="13"/>
+    <row r="583" ht="13"/>
+    <row r="584" ht="13"/>
+    <row r="585" ht="13"/>
+    <row r="586" ht="13"/>
+    <row r="587" ht="13"/>
+    <row r="588" ht="13"/>
+    <row r="589" ht="13"/>
+    <row r="590" ht="13"/>
+    <row r="591" ht="13"/>
+    <row r="592" ht="13"/>
+    <row r="593" ht="13"/>
+    <row r="594" ht="13"/>
+    <row r="595" ht="13"/>
+    <row r="596" ht="13"/>
+    <row r="597" ht="13"/>
+    <row r="598" ht="13"/>
+    <row r="599" ht="13"/>
+    <row r="600" ht="13"/>
+    <row r="601" ht="13"/>
+    <row r="602" ht="13"/>
+    <row r="603" ht="13"/>
+    <row r="604" ht="13"/>
+    <row r="605" ht="13"/>
+    <row r="606" ht="13"/>
+    <row r="607" ht="13"/>
+    <row r="608" ht="13"/>
+    <row r="609" ht="13"/>
+    <row r="610" ht="13"/>
+    <row r="611" ht="13"/>
+    <row r="612" ht="13"/>
+    <row r="613" ht="13"/>
+    <row r="614" ht="13"/>
+    <row r="615" ht="13"/>
+    <row r="616" ht="13"/>
+    <row r="617" ht="13"/>
+    <row r="618" ht="13"/>
+    <row r="619" ht="13"/>
+    <row r="620" ht="13"/>
+    <row r="621" ht="13"/>
+    <row r="622" ht="13"/>
+    <row r="623" ht="13"/>
+    <row r="624" ht="13"/>
+    <row r="625" ht="13"/>
+    <row r="626" ht="13"/>
+    <row r="627" ht="13"/>
+    <row r="628" ht="13"/>
+    <row r="629" ht="13"/>
+    <row r="630" ht="13"/>
+    <row r="631" ht="13"/>
+    <row r="632" ht="13"/>
+    <row r="633" ht="13"/>
+    <row r="634" ht="13"/>
+    <row r="635" ht="13"/>
+    <row r="636" ht="13"/>
+    <row r="637" ht="13"/>
+    <row r="638" ht="13"/>
+    <row r="639" ht="13"/>
+    <row r="640" ht="13"/>
+    <row r="641" ht="13"/>
+    <row r="642" ht="13"/>
+    <row r="643" ht="13"/>
+    <row r="644" ht="13"/>
+    <row r="645" ht="13"/>
+    <row r="646" ht="13"/>
+    <row r="647" ht="13"/>
+    <row r="648" ht="13"/>
+    <row r="649" ht="13"/>
+    <row r="650" ht="13"/>
+    <row r="651" ht="13"/>
+    <row r="652" ht="13"/>
+    <row r="653" ht="13"/>
+    <row r="654" ht="13"/>
+    <row r="655" ht="13"/>
+    <row r="656" ht="13"/>
+    <row r="657" ht="13"/>
+    <row r="658" ht="13"/>
+    <row r="659" ht="13"/>
+    <row r="660" ht="13"/>
+    <row r="661" ht="13"/>
+    <row r="662" ht="13"/>
+    <row r="663" ht="13"/>
+    <row r="664" ht="13"/>
+    <row r="665" ht="13"/>
+    <row r="666" ht="13"/>
+    <row r="667" ht="13"/>
+    <row r="668" ht="13"/>
+    <row r="669" ht="13"/>
+    <row r="670" ht="13"/>
+    <row r="671" ht="13"/>
+    <row r="672" ht="13"/>
+    <row r="673" ht="13"/>
+    <row r="674" ht="13"/>
+    <row r="675" ht="13"/>
+    <row r="676" ht="13"/>
+    <row r="677" ht="13"/>
+    <row r="678" ht="13"/>
+    <row r="679" ht="13"/>
+    <row r="680" ht="13"/>
+    <row r="681" ht="13"/>
+    <row r="682" ht="13"/>
+    <row r="683" ht="13"/>
+    <row r="684" ht="13"/>
+    <row r="685" ht="13"/>
+    <row r="686" ht="13"/>
+    <row r="687" ht="13"/>
+    <row r="688" ht="13"/>
+    <row r="689" ht="13"/>
+    <row r="690" ht="13"/>
+    <row r="691" ht="13"/>
+    <row r="692" ht="13"/>
+    <row r="693" ht="13"/>
+    <row r="694" ht="13"/>
+    <row r="695" ht="13"/>
+    <row r="696" ht="13"/>
+    <row r="697" ht="13"/>
+    <row r="698" ht="13"/>
+    <row r="699" ht="13"/>
+    <row r="700" ht="13"/>
+    <row r="701" ht="13"/>
+    <row r="702" ht="13"/>
+    <row r="703" ht="13"/>
+    <row r="704" ht="13"/>
+    <row r="705" ht="13"/>
+    <row r="706" ht="13"/>
+    <row r="707" ht="13"/>
+    <row r="708" ht="13"/>
+    <row r="709" ht="13"/>
+    <row r="710" ht="13"/>
+    <row r="711" ht="13"/>
+    <row r="712" ht="13"/>
+    <row r="713" ht="13"/>
+    <row r="714" ht="13"/>
+    <row r="715" ht="13"/>
+    <row r="716" ht="13"/>
+    <row r="717" ht="13"/>
+    <row r="718" ht="13"/>
+    <row r="719" ht="13"/>
+    <row r="720" ht="13"/>
+    <row r="721" ht="13"/>
+    <row r="722" ht="13"/>
+    <row r="723" ht="13"/>
+    <row r="724" ht="13"/>
+    <row r="725" ht="13"/>
+    <row r="726" ht="13"/>
+    <row r="727" ht="13"/>
+    <row r="728" ht="13"/>
+    <row r="729" ht="13"/>
+    <row r="730" ht="13"/>
+    <row r="731" ht="13"/>
+    <row r="732" ht="13"/>
+    <row r="733" ht="13"/>
+    <row r="734" ht="13"/>
+    <row r="735" ht="13"/>
+    <row r="736" ht="13"/>
+    <row r="737" ht="13"/>
+    <row r="738" ht="13"/>
+    <row r="739" ht="13"/>
+    <row r="740" ht="13"/>
+    <row r="741" ht="13"/>
+    <row r="742" ht="13"/>
+    <row r="743" ht="13"/>
+    <row r="744" ht="13"/>
+    <row r="745" ht="13"/>
+    <row r="746" ht="13"/>
+    <row r="747" ht="13"/>
+    <row r="748" ht="13"/>
+    <row r="749" ht="13"/>
+    <row r="750" ht="13"/>
+    <row r="751" ht="13"/>
+    <row r="752" ht="13"/>
+    <row r="753" ht="13"/>
+    <row r="754" ht="13"/>
+    <row r="755" ht="13"/>
+    <row r="756" ht="13"/>
+    <row r="757" ht="13"/>
+    <row r="758" ht="13"/>
+    <row r="759" ht="13"/>
+    <row r="760" ht="13"/>
+    <row r="761" ht="13"/>
+    <row r="762" ht="13"/>
+    <row r="763" ht="13"/>
+    <row r="764" ht="13"/>
+    <row r="765" ht="13"/>
+    <row r="766" ht="13"/>
+    <row r="767" ht="13"/>
+    <row r="768" ht="13"/>
+    <row r="769" ht="13"/>
+    <row r="770" ht="13"/>
+    <row r="771" ht="13"/>
+    <row r="772" ht="13"/>
+    <row r="773" ht="13"/>
+    <row r="774" ht="13"/>
+    <row r="775" ht="13"/>
+    <row r="776" ht="13"/>
+    <row r="777" ht="13"/>
+    <row r="778" ht="13"/>
+    <row r="779" ht="13"/>
+    <row r="780" ht="13"/>
+    <row r="781" ht="13"/>
+    <row r="782" ht="13"/>
+    <row r="783" ht="13"/>
+    <row r="784" ht="13"/>
+    <row r="785" ht="13"/>
+    <row r="786" ht="13"/>
+    <row r="787" ht="13"/>
+    <row r="788" ht="13"/>
+    <row r="789" ht="13"/>
+    <row r="790" ht="13"/>
+    <row r="791" ht="13"/>
+    <row r="792" ht="13"/>
+    <row r="793" ht="13"/>
+    <row r="794" ht="13"/>
+    <row r="795" ht="13"/>
+    <row r="796" ht="13"/>
+    <row r="797" ht="13"/>
+    <row r="798" ht="13"/>
+    <row r="799" ht="13"/>
+    <row r="800" ht="13"/>
+    <row r="801" ht="13"/>
+    <row r="802" ht="13"/>
+    <row r="803" ht="13"/>
+    <row r="804" ht="13"/>
+    <row r="805" ht="13"/>
+    <row r="806" ht="13"/>
+    <row r="807" ht="13"/>
+    <row r="808" ht="13"/>
+    <row r="809" ht="13"/>
+    <row r="810" ht="13"/>
+    <row r="811" ht="13"/>
+    <row r="812" ht="13"/>
+    <row r="813" ht="13"/>
+    <row r="814" ht="13"/>
+    <row r="815" ht="13"/>
+    <row r="816" ht="13"/>
+    <row r="817" ht="13"/>
+    <row r="818" ht="13"/>
+    <row r="819" ht="13"/>
+    <row r="820" ht="13"/>
+    <row r="821" ht="13"/>
+    <row r="822" ht="13"/>
+    <row r="823" ht="13"/>
+    <row r="824" ht="13"/>
+    <row r="825" ht="13"/>
+    <row r="826" ht="13"/>
+    <row r="827" ht="13"/>
+    <row r="828" ht="13"/>
+    <row r="829" ht="13"/>
+    <row r="830" ht="13"/>
+    <row r="831" ht="13"/>
+    <row r="832" ht="13"/>
+    <row r="833" ht="13"/>
+    <row r="834" ht="13"/>
+    <row r="835" ht="13"/>
+    <row r="836" ht="13"/>
+    <row r="837" ht="13"/>
+    <row r="838" ht="13"/>
+    <row r="839" ht="13"/>
+    <row r="840" ht="13"/>
+    <row r="841" ht="13"/>
+    <row r="842" ht="13"/>
+    <row r="843" ht="13"/>
+    <row r="844" ht="13"/>
+    <row r="845" ht="13"/>
+    <row r="846" ht="13"/>
+    <row r="847" ht="13"/>
+    <row r="848" ht="13"/>
+    <row r="849" ht="13"/>
+    <row r="850" ht="13"/>
+    <row r="851" ht="13"/>
+    <row r="852" ht="13"/>
+    <row r="853" ht="13"/>
+    <row r="854" ht="13"/>
+    <row r="855" ht="13"/>
+    <row r="856" ht="13"/>
+    <row r="857" ht="13"/>
+    <row r="858" ht="13"/>
+    <row r="859" ht="13"/>
+    <row r="860" ht="13"/>
+    <row r="861" ht="13"/>
+    <row r="862" ht="13"/>
+    <row r="863" ht="13"/>
+    <row r="864" ht="13"/>
+    <row r="865" ht="13"/>
+    <row r="866" ht="13"/>
+    <row r="867" ht="13"/>
+    <row r="868" ht="13"/>
+    <row r="869" ht="13"/>
+    <row r="870" ht="13"/>
+    <row r="871" ht="13"/>
+    <row r="872" ht="13"/>
+    <row r="873" ht="13"/>
+    <row r="874" ht="13"/>
+    <row r="875" ht="13"/>
+    <row r="876" ht="13"/>
+    <row r="877" ht="13"/>
+    <row r="878" ht="13"/>
+    <row r="879" ht="13"/>
+    <row r="880" ht="13"/>
+    <row r="881" ht="13"/>
+    <row r="882" ht="13"/>
+    <row r="883" ht="13"/>
+    <row r="884" ht="13"/>
+    <row r="885" ht="13"/>
+    <row r="886" ht="13"/>
+    <row r="887" ht="13"/>
+    <row r="888" ht="13"/>
+    <row r="889" ht="13"/>
+    <row r="890" ht="13"/>
+    <row r="891" ht="13"/>
+    <row r="892" ht="13"/>
+    <row r="893" ht="13"/>
+    <row r="894" ht="13"/>
+    <row r="895" ht="13"/>
+    <row r="896" ht="13"/>
+    <row r="897" ht="13"/>
+    <row r="898" ht="13"/>
+    <row r="899" ht="13"/>
+    <row r="900" ht="13"/>
+    <row r="901" ht="13"/>
+    <row r="902" ht="13"/>
+    <row r="903" ht="13"/>
+    <row r="904" ht="13"/>
+    <row r="905" ht="13"/>
+    <row r="906" ht="13"/>
+    <row r="907" ht="13"/>
+    <row r="908" ht="13"/>
+    <row r="909" ht="13"/>
+    <row r="910" ht="13"/>
+    <row r="911" ht="13"/>
+    <row r="912" ht="13"/>
+    <row r="913" ht="13"/>
+    <row r="914" ht="13"/>
+    <row r="915" ht="13"/>
+    <row r="916" ht="13"/>
+    <row r="917" ht="13"/>
+    <row r="918" ht="13"/>
+    <row r="919" ht="13"/>
+    <row r="920" ht="13"/>
+    <row r="921" ht="13"/>
+    <row r="922" ht="13"/>
+    <row r="923" ht="13"/>
+    <row r="924" ht="13"/>
+    <row r="925" ht="13"/>
+    <row r="926" ht="13"/>
+    <row r="927" ht="13"/>
+    <row r="928" ht="13"/>
+    <row r="929" ht="13"/>
+    <row r="930" ht="13"/>
+    <row r="931" ht="13"/>
+    <row r="932" ht="13"/>
+    <row r="933" ht="13"/>
+    <row r="934" ht="13"/>
+    <row r="935" ht="13"/>
+    <row r="936" ht="13"/>
+    <row r="937" ht="13"/>
+    <row r="938" ht="13"/>
+    <row r="939" ht="13"/>
+    <row r="940" ht="13"/>
+    <row r="941" ht="13"/>
+    <row r="942" ht="13"/>
+    <row r="943" ht="13"/>
+    <row r="944" ht="13"/>
+    <row r="945" ht="13"/>
+    <row r="946" ht="13"/>
+    <row r="947" ht="13"/>
+    <row r="948" ht="13"/>
+    <row r="949" ht="13"/>
+    <row r="950" ht="13"/>
+    <row r="951" ht="13"/>
+    <row r="952" ht="13"/>
+    <row r="953" ht="13"/>
+    <row r="954" ht="13"/>
+    <row r="955" ht="13"/>
+    <row r="956" ht="13"/>
+    <row r="957" ht="13"/>
+    <row r="958" ht="13"/>
+    <row r="959" ht="13"/>
+    <row r="960" ht="13"/>
+    <row r="961" ht="13"/>
+    <row r="962" ht="13"/>
+    <row r="963" ht="13"/>
+    <row r="964" ht="13"/>
+    <row r="965" ht="13"/>
+    <row r="966" ht="13"/>
+    <row r="967" ht="13"/>
+    <row r="968" ht="13"/>
+    <row r="969" ht="13"/>
+    <row r="970" ht="13"/>
+    <row r="971" ht="13"/>
+    <row r="972" ht="13"/>
+    <row r="973" ht="13"/>
+    <row r="974" ht="13"/>
+    <row r="975" ht="13"/>
+    <row r="976" ht="13"/>
+    <row r="977" ht="13"/>
+    <row r="978" ht="13"/>
+    <row r="979" ht="13"/>
+    <row r="980" ht="13"/>
+    <row r="981" ht="13"/>
+    <row r="982" ht="13"/>
+    <row r="983" ht="13"/>
+    <row r="984" ht="13"/>
+    <row r="985" ht="13"/>
+    <row r="986" ht="13"/>
+    <row r="987" ht="13"/>
+    <row r="988" ht="13"/>
+    <row r="989" ht="13"/>
+    <row r="990" ht="13"/>
+    <row r="991" ht="13"/>
+    <row r="992" ht="13"/>
+    <row r="993" ht="13"/>
+    <row r="994" ht="13"/>
+    <row r="995" ht="13"/>
+    <row r="996" ht="13"/>
+    <row r="997" ht="13"/>
+    <row r="998" ht="13"/>
+    <row r="999" ht="13"/>
+    <row r="1000" ht="13"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:C53"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="30.0"/>
-    <col customWidth="1" min="2" max="2" width="29.13"/>
-    <col customWidth="1" min="3" max="3" width="131.88"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="29.1640625" customWidth="1"/>
+    <col min="3" max="3" width="131.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -4059,7 +4117,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -4070,7 +4128,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3">
       <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
@@ -4081,7 +4139,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -4092,7 +4150,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
@@ -4103,7 +4161,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3">
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
@@ -4114,7 +4172,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
@@ -4125,7 +4183,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
@@ -4136,7 +4194,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
         <v>9</v>
       </c>
@@ -4147,7 +4205,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
@@ -4158,7 +4216,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
         <v>11</v>
       </c>
@@ -4169,7 +4227,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -4180,7 +4238,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3">
       <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
@@ -4191,7 +4249,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:3">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -4202,7 +4260,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:3">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -4213,7 +4271,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:3">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
@@ -4224,7 +4282,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3">
       <c r="A17" s="5" t="s">
         <v>17</v>
       </c>
@@ -4235,7 +4293,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3">
       <c r="A18" s="5" t="s">
         <v>18</v>
       </c>
@@ -4246,7 +4304,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:3">
       <c r="A19" s="5" t="s">
         <v>19</v>
       </c>
@@ -4257,7 +4315,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3">
       <c r="A20" s="5" t="s">
         <v>20</v>
       </c>
@@ -4268,7 +4326,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:3">
       <c r="A21" s="5" t="s">
         <v>21</v>
       </c>
@@ -4279,7 +4337,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:3">
       <c r="A22" s="5" t="s">
         <v>22</v>
       </c>
@@ -4290,7 +4348,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:3">
       <c r="A23" s="5" t="s">
         <v>23</v>
       </c>
@@ -4301,7 +4359,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:3">
       <c r="A24" s="5" t="s">
         <v>24</v>
       </c>
@@ -4312,7 +4370,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:3">
       <c r="A25" s="5" t="s">
         <v>25</v>
       </c>
@@ -4323,7 +4381,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:3">
       <c r="A26" s="5" t="s">
         <v>26</v>
       </c>
@@ -4334,7 +4392,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:3">
       <c r="A27" s="5" t="s">
         <v>28</v>
       </c>
@@ -4345,7 +4403,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:3">
       <c r="A28" s="5" t="s">
         <v>29</v>
       </c>
@@ -4356,7 +4414,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:3">
       <c r="A29" s="5" t="s">
         <v>30</v>
       </c>
@@ -4367,7 +4425,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:3">
       <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
@@ -4378,7 +4436,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:3">
       <c r="A31" s="5" t="s">
         <v>32</v>
       </c>
@@ -4389,7 +4447,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:3">
       <c r="A32" s="5" t="s">
         <v>34</v>
       </c>
@@ -4400,7 +4458,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:3">
       <c r="A33" s="5" t="s">
         <v>36</v>
       </c>
@@ -4411,7 +4469,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:3">
       <c r="A34" s="5" t="s">
         <v>37</v>
       </c>
@@ -4422,7 +4480,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:3">
       <c r="A35" s="5" t="s">
         <v>38</v>
       </c>
@@ -4433,7 +4491,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:3">
       <c r="A36" s="5" t="s">
         <v>39</v>
       </c>
@@ -4444,7 +4502,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:3">
       <c r="A37" s="5" t="s">
         <v>40</v>
       </c>
@@ -4455,7 +4513,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:3">
       <c r="A38" s="5" t="s">
         <v>41</v>
       </c>
@@ -4466,7 +4524,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:3">
       <c r="A39" s="5" t="s">
         <v>42</v>
       </c>
@@ -4477,117 +4535,127 @@
         <v>190</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="13"/>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-    </row>
-    <row r="41">
+    <row r="40" spans="1:3">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41" s="3" t="s">
         <v>195</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="C41" s="13"/>
-    </row>
-    <row r="42">
+      <c r="C41" s="5"/>
+    </row>
+    <row r="42" spans="1:3">
       <c r="A42" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="17" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="43">
+      <c r="C42" s="18"/>
+    </row>
+    <row r="43" spans="1:3">
       <c r="A43" s="5" t="s">
         <v>201</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C43" s="13"/>
-    </row>
-    <row r="44">
+      <c r="C43" s="5"/>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44" s="5" t="s">
         <v>203</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="C44" s="13"/>
-    </row>
-    <row r="45">
+      <c r="C44" s="5"/>
+    </row>
+    <row r="45" spans="1:3">
       <c r="A45" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="17" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="46">
+      <c r="C45" s="18"/>
+    </row>
+    <row r="46" spans="1:3">
       <c r="A46" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="17" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="47">
+      <c r="C46" s="18"/>
+    </row>
+    <row r="47" spans="1:3">
       <c r="A47" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="17" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="48">
+      <c r="C47" s="18"/>
+    </row>
+    <row r="48" spans="1:3">
       <c r="A48" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="17" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="49">
+      <c r="C48" s="18"/>
+    </row>
+    <row r="49" spans="1:3">
       <c r="A49" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="17" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="50">
+      <c r="C49" s="18"/>
+    </row>
+    <row r="50" spans="1:3">
       <c r="A50" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="17" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="51">
+      <c r="C50" s="18"/>
+    </row>
+    <row r="51" spans="1:3">
       <c r="A51" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="17" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="52">
+      <c r="C51" s="18"/>
+    </row>
+    <row r="52" spans="1:3">
       <c r="A52" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="17" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="53">
+      <c r="C52" s="18"/>
+    </row>
+    <row r="53" spans="1:3">
       <c r="A53" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="17" t="s">
         <v>233</v>
       </c>
+      <c r="C53" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -4602,221 +4670,222 @@
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="B50:C50"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:A79"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="132.5"/>
+    <col min="1" max="1" width="132.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="s">
+    <row r="7" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A7" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="s">
+    <row r="9" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A9" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="s">
+    <row r="11" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A11" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A13" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A15" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A17" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="s">
+    <row r="19" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A19" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A21" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="s">
+    <row r="23" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A23" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="9" t="s">
+    <row r="25" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A25" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="s">
+    <row r="27" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A27" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="9" t="s">
+    <row r="29" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A29" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="9" t="s">
+    <row r="31" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A31" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="9" t="s">
+    <row r="33" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A33" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="9" t="s">
+    <row r="35" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A35" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="9" t="s">
+    <row r="37" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A37" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="9" t="s">
+    <row r="39" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A39" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="9" t="s">
+    <row r="41" spans="1:1" ht="15.75" customHeight="1">
+      <c r="A41" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="9" t="s">
+    <row r="43" spans="1:1" ht="13">
+      <c r="A43" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="9" t="s">
+    <row r="45" spans="1:1" ht="13">
+      <c r="A45" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="9" t="s">
+    <row r="47" spans="1:1" ht="13">
+      <c r="A47" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="9" t="s">
+    <row r="49" spans="1:1" ht="13">
+      <c r="A49" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="9" t="s">
+    <row r="51" spans="1:1" ht="13">
+      <c r="A51" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="9" t="s">
+    <row r="53" spans="1:1" ht="13">
+      <c r="A53" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="9" t="s">
+    <row r="55" spans="1:1" ht="13">
+      <c r="A55" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="9" t="s">
+    <row r="57" spans="1:1" ht="13">
+      <c r="A57" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="9" t="s">
+    <row r="59" spans="1:1" ht="13">
+      <c r="A59" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="9" t="s">
+    <row r="61" spans="1:1" ht="13">
+      <c r="A61" s="1" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="9" t="s">
+    <row r="63" spans="1:1" ht="13">
+      <c r="A63" s="1" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="9" t="s">
+    <row r="65" spans="1:1" ht="13">
+      <c r="A65" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="9" t="s">
+    <row r="67" spans="1:1" ht="13">
+      <c r="A67" s="1" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="9" t="s">
+    <row r="69" spans="1:1" ht="13">
+      <c r="A69" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="9" t="s">
+    <row r="71" spans="1:1" ht="13">
+      <c r="A71" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="9" t="s">
+    <row r="73" spans="1:1" ht="13">
+      <c r="A73" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="9" t="s">
+    <row r="75" spans="1:1" ht="13">
+      <c r="A75" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="9" t="s">
+    <row r="77" spans="1:1" ht="13">
+      <c r="A77" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="9" t="s">
+    <row r="79" spans="1:1" ht="13">
+      <c r="A79" s="1" t="s">
         <v>186</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>